<commit_message>
Unify Research Hub demo on canonical S&P 500 top 100
</commit_message>
<xml_diff>
--- a/public/portfolio/portfolio-demo-100.xlsx
+++ b/public/portfolio/portfolio-demo-100.xlsx
@@ -117,7 +117,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AAPL</t>
+          <t xml:space="preserve">NVDA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001045810</t>
         </is>
       </c>
       <c r="E2">
@@ -127,7 +132,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MSFT</t>
+          <t xml:space="preserve">AAPL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000320193</t>
         </is>
       </c>
       <c r="E3">
@@ -137,87 +147,132 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NVDA</t>
+          <t xml:space="preserve">MSFT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000789019</t>
         </is>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORCL</t>
+          <t xml:space="preserve">GOOGL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001652044</t>
         </is>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADBE</t>
+          <t xml:space="preserve">AMZN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001018724</t>
         </is>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRM</t>
+          <t xml:space="preserve">AVGO</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001730168</t>
         </is>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD</t>
+          <t xml:space="preserve">META</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001326801</t>
         </is>
       </c>
       <c r="E8">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTC</t>
+          <t xml:space="preserve">MU</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000723125</t>
         </is>
       </c>
       <c r="E9">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">CSCO</t>
+          <t xml:space="preserve">TSLA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001318605</t>
         </is>
       </c>
       <c r="E10">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">IBM</t>
+          <t xml:space="preserve">JPM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000019617</t>
         </is>
       </c>
       <c r="E11">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMZN</t>
+          <t xml:space="preserve">BRK-B</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001067983</t>
         </is>
       </c>
       <c r="E12">
@@ -227,127 +282,192 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">TSLA</t>
+          <t xml:space="preserve">LLY</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000059478</t>
         </is>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">HD</t>
+          <t xml:space="preserve">AMD</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000002488</t>
         </is>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">LOW</t>
+          <t xml:space="preserve">XOM</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0002115436</t>
         </is>
       </c>
       <c r="E15">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">NKE</t>
+          <t xml:space="preserve">JNJ</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000200406</t>
         </is>
       </c>
       <c r="E16">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCD</t>
+          <t xml:space="preserve">V</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001403161</t>
         </is>
       </c>
       <c r="E17">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">SBUX</t>
+          <t xml:space="preserve">INTC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000050863</t>
         </is>
       </c>
       <c r="E18">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">TGT</t>
+          <t xml:space="preserve">WMT</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000104169</t>
         </is>
       </c>
       <c r="E19">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">TJX</t>
+          <t xml:space="preserve">MA</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001141391</t>
         </is>
       </c>
       <c r="E20">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">BKNG</t>
+          <t xml:space="preserve">ABBV</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001551152</t>
         </is>
       </c>
       <c r="E21">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">WMT</t>
+          <t xml:space="preserve">CSCO</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000858877</t>
         </is>
       </c>
       <c r="E22">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">COST</t>
+          <t xml:space="preserve">BAC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000070858</t>
         </is>
       </c>
       <c r="E23">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">PG</t>
+          <t xml:space="preserve">COST</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000909832</t>
         </is>
       </c>
       <c r="E24">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CVX</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000093410</t>
         </is>
       </c>
       <c r="E25">
@@ -357,7 +477,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEP</t>
+          <t xml:space="preserve">PLTR</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001321655</t>
         </is>
       </c>
       <c r="E26">
@@ -367,7 +492,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDLZ</t>
+          <t xml:space="preserve">CAT</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000018230</t>
         </is>
       </c>
       <c r="E27">
@@ -377,67 +507,102 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">CL</t>
+          <t xml:space="preserve">LRCX</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000707549</t>
         </is>
       </c>
       <c r="E28">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">KMB</t>
+          <t xml:space="preserve">AMAT</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000006951</t>
         </is>
       </c>
       <c r="E29">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">GIS</t>
+          <t xml:space="preserve">MRK</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000310158</t>
         </is>
       </c>
       <c r="E30">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">KHC</t>
+          <t xml:space="preserve">UNH</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000731766</t>
         </is>
       </c>
       <c r="E31">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">JPM</t>
+          <t xml:space="preserve">KO</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000021344</t>
         </is>
       </c>
       <c r="E32">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">BAC</t>
+          <t xml:space="preserve">PG</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000080424</t>
         </is>
       </c>
       <c r="E33">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">WFC</t>
+          <t xml:space="preserve">GE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000040545</t>
         </is>
       </c>
       <c r="E34">
@@ -447,7 +612,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">NFLX</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001065280</t>
         </is>
       </c>
       <c r="E35">
@@ -457,7 +627,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">GS</t>
+          <t xml:space="preserve">HD</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000354950</t>
         </is>
       </c>
       <c r="E36">
@@ -467,77 +642,117 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">MS</t>
+          <t xml:space="preserve">GS</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000886982</t>
         </is>
       </c>
       <c r="E37">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">AXP</t>
+          <t xml:space="preserve">PM</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001413329</t>
         </is>
       </c>
       <c r="E38">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">SCHW</t>
+          <t xml:space="preserve">WFC</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000072971</t>
         </is>
       </c>
       <c r="E39">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">USB</t>
+          <t xml:space="preserve">PANW</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001327567</t>
         </is>
       </c>
       <c r="E40">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">PNC</t>
+          <t xml:space="preserve">RTX</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000101829</t>
         </is>
       </c>
       <c r="E41">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNH</t>
+          <t xml:space="preserve">GEV</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001996810</t>
         </is>
       </c>
       <c r="E42">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">JNJ</t>
+          <t xml:space="preserve">MS</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000895421</t>
         </is>
       </c>
       <c r="E43">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">LLY</t>
+          <t xml:space="preserve">ORCL</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001341439</t>
         </is>
       </c>
       <c r="E44">
@@ -547,7 +762,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">MRK</t>
+          <t xml:space="preserve">TXN</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000097476</t>
         </is>
       </c>
       <c r="E45">
@@ -557,7 +777,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">ABBV</t>
+          <t xml:space="preserve">SNDK</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0002023554</t>
         </is>
       </c>
       <c r="E46">
@@ -567,97 +792,147 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">ABT</t>
+          <t xml:space="preserve">C</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000831001</t>
         </is>
       </c>
       <c r="E47">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">TMO</t>
+          <t xml:space="preserve">KLAC</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000319201</t>
         </is>
       </c>
       <c r="E48">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">DHR</t>
+          <t xml:space="preserve">IBM</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000051143</t>
         </is>
       </c>
       <c r="E49">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMGN</t>
+          <t xml:space="preserve">TMO</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000097745</t>
         </is>
       </c>
       <c r="E50">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">GILD</t>
+          <t xml:space="preserve">LIN</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001707925</t>
         </is>
       </c>
       <c r="E51">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAT</t>
+          <t xml:space="preserve">VZ</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000732712</t>
         </is>
       </c>
       <c r="E52">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">DE</t>
+          <t xml:space="preserve">CRWD</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001535527</t>
         </is>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE</t>
+          <t xml:space="preserve">MRVL</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001835632</t>
         </is>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">HON</t>
+          <t xml:space="preserve">APH</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000820313</t>
         </is>
       </c>
       <c r="E55">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">UPS</t>
+          <t xml:space="preserve">ANET</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001596532</t>
         </is>
       </c>
       <c r="E56">
@@ -667,7 +942,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">FDX</t>
+          <t xml:space="preserve">AMGN</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000318154</t>
         </is>
       </c>
       <c r="E57">
@@ -677,17 +957,27 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">RTX</t>
+          <t xml:space="preserve">CRM</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001108524</t>
         </is>
       </c>
       <c r="E58">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">LMT</t>
+          <t xml:space="preserve">QCOM</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000804328</t>
         </is>
       </c>
       <c r="E59">
@@ -697,7 +987,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">NOC</t>
+          <t xml:space="preserve">PEP</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000077476</t>
         </is>
       </c>
       <c r="E60">
@@ -707,7 +1002,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">GD</t>
+          <t xml:space="preserve">STX</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001137789</t>
         </is>
       </c>
       <c r="E61">
@@ -717,57 +1017,87 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">XOM</t>
+          <t xml:space="preserve">DIS</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001744489</t>
         </is>
       </c>
       <c r="E62">
-        <v>5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">CVX</t>
+          <t xml:space="preserve">ADI</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000006281</t>
         </is>
       </c>
       <c r="E63">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">COP</t>
+          <t xml:space="preserve">T</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000732717</t>
         </is>
       </c>
       <c r="E64">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">EOG</t>
+          <t xml:space="preserve">MCD</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000063908</t>
         </is>
       </c>
       <c r="E65">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">SLB</t>
+          <t xml:space="preserve">GILD</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000882095</t>
         </is>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">OXY</t>
+          <t xml:space="preserve">ABT</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000001800</t>
         </is>
       </c>
       <c r="E67">
@@ -777,7 +1107,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSX</t>
+          <t xml:space="preserve">SCHW</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000316709</t>
         </is>
       </c>
       <c r="E68">
@@ -787,7 +1122,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">VLO</t>
+          <t xml:space="preserve">AXP</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000004962</t>
         </is>
       </c>
       <c r="E69">
@@ -797,7 +1137,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">MPC</t>
+          <t xml:space="preserve">NEE</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000753308</t>
         </is>
       </c>
       <c r="E70">
@@ -807,7 +1152,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">KMI</t>
+          <t xml:space="preserve">DE</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000315189</t>
         </is>
       </c>
       <c r="E71">
@@ -817,47 +1167,72 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">NEE</t>
+          <t xml:space="preserve">UNP</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000100885</t>
         </is>
       </c>
       <c r="E72">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">DUK</t>
+          <t xml:space="preserve">COP</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001163165</t>
         </is>
       </c>
       <c r="E73">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">SO</t>
+          <t xml:space="preserve">WELL</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000766704</t>
         </is>
       </c>
       <c r="E74">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">AEP</t>
+          <t xml:space="preserve">BA</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000012927</t>
         </is>
       </c>
       <c r="E75">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXC</t>
+          <t xml:space="preserve">ETN</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001551182</t>
         </is>
       </c>
       <c r="E76">
@@ -867,7 +1242,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRE</t>
+          <t xml:space="preserve">DELL</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001571996</t>
         </is>
       </c>
       <c r="E77">
@@ -877,7 +1257,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">XEL</t>
+          <t xml:space="preserve">PFE</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000078003</t>
         </is>
       </c>
       <c r="E78">
@@ -887,7 +1272,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">WEC</t>
+          <t xml:space="preserve">BLK</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0002012383</t>
         </is>
       </c>
       <c r="E79">
@@ -897,7 +1287,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">ED</t>
+          <t xml:space="preserve">WDC</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000106040</t>
         </is>
       </c>
       <c r="E80">
@@ -907,7 +1302,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">D</t>
+          <t xml:space="preserve">UBER</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001543151</t>
         </is>
       </c>
       <c r="E81">
@@ -917,57 +1317,87 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">GOOGL</t>
+          <t xml:space="preserve">TJX</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000109198</t>
         </is>
       </c>
       <c r="E82">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">META</t>
+          <t xml:space="preserve">NOW</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001373715</t>
         </is>
       </c>
       <c r="E83">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">NFLX</t>
+          <t xml:space="preserve">NEM</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001164727</t>
         </is>
       </c>
       <c r="E84">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">DIS</t>
+          <t xml:space="preserve">BKNG</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001075531</t>
         </is>
       </c>
       <c r="E85">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">CMCSA</t>
+          <t xml:space="preserve">VRTX</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000875320</t>
         </is>
       </c>
       <c r="E86">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">VZ</t>
+          <t xml:space="preserve">ISRG</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001035267</t>
         </is>
       </c>
       <c r="E87">
@@ -977,7 +1407,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">T</t>
+          <t xml:space="preserve">GLW</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000024741</t>
         </is>
       </c>
       <c r="E88">
@@ -987,7 +1422,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">CHTR</t>
+          <t xml:space="preserve">BMY</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000014272</t>
         </is>
       </c>
       <c r="E89">
@@ -997,7 +1437,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">TTWO</t>
+          <t xml:space="preserve">COF</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000927628</t>
         </is>
       </c>
       <c r="E90">
@@ -1007,7 +1452,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">WBD</t>
+          <t xml:space="preserve">PLD</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001045609</t>
         </is>
       </c>
       <c r="E91">
@@ -1017,37 +1467,57 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">LIN</t>
+          <t xml:space="preserve">PGR</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000080661</t>
         </is>
       </c>
       <c r="E92">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">APD</t>
+          <t xml:space="preserve">DHR</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000313616</t>
         </is>
       </c>
       <c r="E93">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHW</t>
+          <t xml:space="preserve">SPGI</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000064040</t>
         </is>
       </c>
       <c r="E94">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">FCX</t>
+          <t xml:space="preserve">CB</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000896159</t>
         </is>
       </c>
       <c r="E95">
@@ -1057,7 +1527,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">NEM</t>
+          <t xml:space="preserve">CVS</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000064803</t>
         </is>
       </c>
       <c r="E96">
@@ -1067,7 +1542,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">NUE</t>
+          <t xml:space="preserve">PH</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000076334</t>
         </is>
       </c>
       <c r="E97">
@@ -1077,27 +1557,42 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLD</t>
+          <t xml:space="preserve">MDT</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001613103</t>
         </is>
       </c>
       <c r="E98">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMT</t>
+          <t xml:space="preserve">VLO</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001035002</t>
         </is>
       </c>
       <c r="E99">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPG</t>
+          <t xml:space="preserve">MPC</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001510295</t>
         </is>
       </c>
       <c r="E100">
@@ -1107,7 +1602,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">O</t>
+          <t xml:space="preserve">MO</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000764180</t>
         </is>
       </c>
       <c r="E101">
@@ -1127,7 +1627,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Hypothetical weighted portfolio · 100-company demo</t>
+          <t xml:space="preserve">S&amp;P 500 coverage portfolio · top 100 companies</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1639,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Upload this workbook in Research Hub → Portfolio research. The Holdings sheet contains 100 company tickers and hypothetical weight_pct values totaling 100%. Select Weighted portfolio — supplied weight_pct in Allocation settings after import.</t>
+          <t xml:space="preserve">Upload this workbook in Research Hub → Portfolio research. The Holdings sheet contains 100 company tickers, their verified SEC CIKs and hypothetical weight_pct values totaling 100%. Select Weighted portfolio — supplied weight_pct in Allocation settings after import.</t>
         </is>
       </c>
     </row>
@@ -1163,65 +1663,101 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">This is a selected demonstration list, not an index, a representative market sample, actual holdings or an investment recommendation.</t>
+          <t xml:space="preserve">The 100 largest issuer holdings in the stored S&amp;P 500 coverage list, ranked by combined IVV holding weight as of 2026-09-11. Share classes are combined by SEC issuer. Portfolio allocations are fixed hypothetical examples, independent of IVV weights; this is a dated research demonstration, not an index portfolio or an investment recommendation.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hypothetical weights</t>
+          <t xml:space="preserve">Coverage membership</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed hypothetical weights: 5 companies at 5% each, 15 at 2%, 30 at 1%, and 50 at 0.3%, totaling 100%. These educational inputs are not derived from market prices, company fundamentals, an index, or actual holdings and are not investment recommendations.</t>
+          <t xml:space="preserve">sec-coverage-v1:ivv:2026-09-11:3e50096539317ce6</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Weight units</t>
+          <t xml:space="preserve">Membership source</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">weight_pct uses percentage points: 5 means 5%, and 0.3 means 0.3%. These are literal values. The remaining input fields are blank. Clear the weights to use your own company research list.</t>
+          <t xml:space="preserve">IVV holdings as of 2026-09-11; https://www.ishares.com/us/products/239726/ishares-core-s-p-500-etf/latest-holdings.csv</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dates</t>
+          <t xml:space="preserve">Company selection</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">The example analysis is a dated capture. Running research retrieves current available public evidence; results and coverage may differ.</t>
+          <t xml:space="preserve">The 100 largest issuer holdings in the active IVV S&amp;P 500 coverage source, ranked by combined published fund weight across share classes. Ties use combined holding market value, then ticker. Each SEC issuer appears once, represented by its largest share class. IVV holdings are a dated coverage proxy, not certified current index membership.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Limits</t>
+          <t xml:space="preserve">Hypothetical weights</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">The import supports at most 100 rows. Replace existing tickers before adding more. Cells contain literal values, with no formulas or macros.</t>
+          <t xml:space="preserve">Fixed hypothetical weights by demo order: the first 5 companies receive 5% each, the next 15 receive 2%, the next 30 receive 1%, and the remaining 50 receive 0.3%, totaling 100%. These educational amounts are fixed independently of source fund weights, prices and company fundamentals. They are not actual holdings, index weights or investment recommendations.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t xml:space="preserve">Weight units</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weight_pct uses percentage points: 5 means 5%, and 0.3 means 0.3%. These are literal hypothetical allocations, not the IVV weights used to select companies. Other than ticker, CIK and weight_pct, the input fields are blank. Clear the weights to use company counts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dates</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The example analysis is a dated capture. Running research retrieves current available public evidence; results and coverage may differ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limits</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The import supports at most 100 rows. Replace existing tickers before adding more. Cells contain literal values, with no formulas or macros.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Privacy</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t xml:space="preserve">Imported notes remain in your browser. Interactive research sends company identifiers, not private allocations or notes.</t>
         </is>

</xml_diff>

<commit_message>
Unify Research Hub demo on S&P 500 top 100 and remove Research prompts (#80)
* Unify Research Hub demo on canonical S&P 500 top 100

* Derive demo industry coverage from selected companies
</commit_message>
<xml_diff>
--- a/public/portfolio/portfolio-demo-100.xlsx
+++ b/public/portfolio/portfolio-demo-100.xlsx
@@ -117,7 +117,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AAPL</t>
+          <t xml:space="preserve">NVDA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001045810</t>
         </is>
       </c>
       <c r="E2">
@@ -127,7 +132,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MSFT</t>
+          <t xml:space="preserve">AAPL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000320193</t>
         </is>
       </c>
       <c r="E3">
@@ -137,87 +147,132 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NVDA</t>
+          <t xml:space="preserve">MSFT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000789019</t>
         </is>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORCL</t>
+          <t xml:space="preserve">GOOGL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001652044</t>
         </is>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADBE</t>
+          <t xml:space="preserve">AMZN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001018724</t>
         </is>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRM</t>
+          <t xml:space="preserve">AVGO</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001730168</t>
         </is>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMD</t>
+          <t xml:space="preserve">META</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001326801</t>
         </is>
       </c>
       <c r="E8">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTC</t>
+          <t xml:space="preserve">MU</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000723125</t>
         </is>
       </c>
       <c r="E9">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">CSCO</t>
+          <t xml:space="preserve">TSLA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001318605</t>
         </is>
       </c>
       <c r="E10">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">IBM</t>
+          <t xml:space="preserve">JPM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000019617</t>
         </is>
       </c>
       <c r="E11">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMZN</t>
+          <t xml:space="preserve">BRK-B</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001067983</t>
         </is>
       </c>
       <c r="E12">
@@ -227,127 +282,192 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">TSLA</t>
+          <t xml:space="preserve">LLY</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000059478</t>
         </is>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">HD</t>
+          <t xml:space="preserve">AMD</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000002488</t>
         </is>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">LOW</t>
+          <t xml:space="preserve">XOM</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0002115436</t>
         </is>
       </c>
       <c r="E15">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">NKE</t>
+          <t xml:space="preserve">JNJ</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000200406</t>
         </is>
       </c>
       <c r="E16">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCD</t>
+          <t xml:space="preserve">V</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001403161</t>
         </is>
       </c>
       <c r="E17">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">SBUX</t>
+          <t xml:space="preserve">INTC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000050863</t>
         </is>
       </c>
       <c r="E18">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">TGT</t>
+          <t xml:space="preserve">WMT</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000104169</t>
         </is>
       </c>
       <c r="E19">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">TJX</t>
+          <t xml:space="preserve">MA</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001141391</t>
         </is>
       </c>
       <c r="E20">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">BKNG</t>
+          <t xml:space="preserve">ABBV</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001551152</t>
         </is>
       </c>
       <c r="E21">
-        <v>0.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">WMT</t>
+          <t xml:space="preserve">CSCO</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000858877</t>
         </is>
       </c>
       <c r="E22">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">COST</t>
+          <t xml:space="preserve">BAC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000070858</t>
         </is>
       </c>
       <c r="E23">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">PG</t>
+          <t xml:space="preserve">COST</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000909832</t>
         </is>
       </c>
       <c r="E24">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CVX</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000093410</t>
         </is>
       </c>
       <c r="E25">
@@ -357,7 +477,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEP</t>
+          <t xml:space="preserve">PLTR</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001321655</t>
         </is>
       </c>
       <c r="E26">
@@ -367,7 +492,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDLZ</t>
+          <t xml:space="preserve">CAT</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000018230</t>
         </is>
       </c>
       <c r="E27">
@@ -377,67 +507,102 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">CL</t>
+          <t xml:space="preserve">LRCX</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000707549</t>
         </is>
       </c>
       <c r="E28">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">KMB</t>
+          <t xml:space="preserve">AMAT</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000006951</t>
         </is>
       </c>
       <c r="E29">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">GIS</t>
+          <t xml:space="preserve">MRK</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000310158</t>
         </is>
       </c>
       <c r="E30">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">KHC</t>
+          <t xml:space="preserve">UNH</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000731766</t>
         </is>
       </c>
       <c r="E31">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">JPM</t>
+          <t xml:space="preserve">KO</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000021344</t>
         </is>
       </c>
       <c r="E32">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">BAC</t>
+          <t xml:space="preserve">PG</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000080424</t>
         </is>
       </c>
       <c r="E33">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">WFC</t>
+          <t xml:space="preserve">GE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000040545</t>
         </is>
       </c>
       <c r="E34">
@@ -447,7 +612,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">NFLX</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001065280</t>
         </is>
       </c>
       <c r="E35">
@@ -457,7 +627,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">GS</t>
+          <t xml:space="preserve">HD</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000354950</t>
         </is>
       </c>
       <c r="E36">
@@ -467,77 +642,117 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">MS</t>
+          <t xml:space="preserve">GS</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000886982</t>
         </is>
       </c>
       <c r="E37">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">AXP</t>
+          <t xml:space="preserve">PM</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001413329</t>
         </is>
       </c>
       <c r="E38">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">SCHW</t>
+          <t xml:space="preserve">WFC</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000072971</t>
         </is>
       </c>
       <c r="E39">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">USB</t>
+          <t xml:space="preserve">PANW</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001327567</t>
         </is>
       </c>
       <c r="E40">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">PNC</t>
+          <t xml:space="preserve">RTX</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000101829</t>
         </is>
       </c>
       <c r="E41">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNH</t>
+          <t xml:space="preserve">GEV</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001996810</t>
         </is>
       </c>
       <c r="E42">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">JNJ</t>
+          <t xml:space="preserve">MS</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000895421</t>
         </is>
       </c>
       <c r="E43">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">LLY</t>
+          <t xml:space="preserve">ORCL</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001341439</t>
         </is>
       </c>
       <c r="E44">
@@ -547,7 +762,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">MRK</t>
+          <t xml:space="preserve">TXN</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000097476</t>
         </is>
       </c>
       <c r="E45">
@@ -557,7 +777,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">ABBV</t>
+          <t xml:space="preserve">SNDK</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0002023554</t>
         </is>
       </c>
       <c r="E46">
@@ -567,97 +792,147 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">ABT</t>
+          <t xml:space="preserve">C</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000831001</t>
         </is>
       </c>
       <c r="E47">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">TMO</t>
+          <t xml:space="preserve">KLAC</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000319201</t>
         </is>
       </c>
       <c r="E48">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">DHR</t>
+          <t xml:space="preserve">IBM</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000051143</t>
         </is>
       </c>
       <c r="E49">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMGN</t>
+          <t xml:space="preserve">TMO</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000097745</t>
         </is>
       </c>
       <c r="E50">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">GILD</t>
+          <t xml:space="preserve">LIN</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001707925</t>
         </is>
       </c>
       <c r="E51">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAT</t>
+          <t xml:space="preserve">VZ</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000732712</t>
         </is>
       </c>
       <c r="E52">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">DE</t>
+          <t xml:space="preserve">CRWD</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001535527</t>
         </is>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">GE</t>
+          <t xml:space="preserve">MRVL</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001835632</t>
         </is>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">HON</t>
+          <t xml:space="preserve">APH</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000820313</t>
         </is>
       </c>
       <c r="E55">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">UPS</t>
+          <t xml:space="preserve">ANET</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001596532</t>
         </is>
       </c>
       <c r="E56">
@@ -667,7 +942,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">FDX</t>
+          <t xml:space="preserve">AMGN</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000318154</t>
         </is>
       </c>
       <c r="E57">
@@ -677,17 +957,27 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">RTX</t>
+          <t xml:space="preserve">CRM</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001108524</t>
         </is>
       </c>
       <c r="E58">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">LMT</t>
+          <t xml:space="preserve">QCOM</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000804328</t>
         </is>
       </c>
       <c r="E59">
@@ -697,7 +987,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">NOC</t>
+          <t xml:space="preserve">PEP</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000077476</t>
         </is>
       </c>
       <c r="E60">
@@ -707,7 +1002,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">GD</t>
+          <t xml:space="preserve">STX</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001137789</t>
         </is>
       </c>
       <c r="E61">
@@ -717,57 +1017,87 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">XOM</t>
+          <t xml:space="preserve">DIS</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001744489</t>
         </is>
       </c>
       <c r="E62">
-        <v>5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">CVX</t>
+          <t xml:space="preserve">ADI</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000006281</t>
         </is>
       </c>
       <c r="E63">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">COP</t>
+          <t xml:space="preserve">T</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000732717</t>
         </is>
       </c>
       <c r="E64">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">EOG</t>
+          <t xml:space="preserve">MCD</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000063908</t>
         </is>
       </c>
       <c r="E65">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">SLB</t>
+          <t xml:space="preserve">GILD</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000882095</t>
         </is>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">OXY</t>
+          <t xml:space="preserve">ABT</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000001800</t>
         </is>
       </c>
       <c r="E67">
@@ -777,7 +1107,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSX</t>
+          <t xml:space="preserve">SCHW</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000316709</t>
         </is>
       </c>
       <c r="E68">
@@ -787,7 +1122,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">VLO</t>
+          <t xml:space="preserve">AXP</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000004962</t>
         </is>
       </c>
       <c r="E69">
@@ -797,7 +1137,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">MPC</t>
+          <t xml:space="preserve">NEE</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000753308</t>
         </is>
       </c>
       <c r="E70">
@@ -807,7 +1152,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">KMI</t>
+          <t xml:space="preserve">DE</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000315189</t>
         </is>
       </c>
       <c r="E71">
@@ -817,47 +1167,72 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">NEE</t>
+          <t xml:space="preserve">UNP</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000100885</t>
         </is>
       </c>
       <c r="E72">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">DUK</t>
+          <t xml:space="preserve">COP</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001163165</t>
         </is>
       </c>
       <c r="E73">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">SO</t>
+          <t xml:space="preserve">WELL</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000766704</t>
         </is>
       </c>
       <c r="E74">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">AEP</t>
+          <t xml:space="preserve">BA</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000012927</t>
         </is>
       </c>
       <c r="E75">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXC</t>
+          <t xml:space="preserve">ETN</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001551182</t>
         </is>
       </c>
       <c r="E76">
@@ -867,7 +1242,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRE</t>
+          <t xml:space="preserve">DELL</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001571996</t>
         </is>
       </c>
       <c r="E77">
@@ -877,7 +1257,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">XEL</t>
+          <t xml:space="preserve">PFE</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000078003</t>
         </is>
       </c>
       <c r="E78">
@@ -887,7 +1272,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">WEC</t>
+          <t xml:space="preserve">BLK</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0002012383</t>
         </is>
       </c>
       <c r="E79">
@@ -897,7 +1287,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">ED</t>
+          <t xml:space="preserve">WDC</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000106040</t>
         </is>
       </c>
       <c r="E80">
@@ -907,7 +1302,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">D</t>
+          <t xml:space="preserve">UBER</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001543151</t>
         </is>
       </c>
       <c r="E81">
@@ -917,57 +1317,87 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">GOOGL</t>
+          <t xml:space="preserve">TJX</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000109198</t>
         </is>
       </c>
       <c r="E82">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">META</t>
+          <t xml:space="preserve">NOW</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001373715</t>
         </is>
       </c>
       <c r="E83">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">NFLX</t>
+          <t xml:space="preserve">NEM</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001164727</t>
         </is>
       </c>
       <c r="E84">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">DIS</t>
+          <t xml:space="preserve">BKNG</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001075531</t>
         </is>
       </c>
       <c r="E85">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">CMCSA</t>
+          <t xml:space="preserve">VRTX</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000875320</t>
         </is>
       </c>
       <c r="E86">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">VZ</t>
+          <t xml:space="preserve">ISRG</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001035267</t>
         </is>
       </c>
       <c r="E87">
@@ -977,7 +1407,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">T</t>
+          <t xml:space="preserve">GLW</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000024741</t>
         </is>
       </c>
       <c r="E88">
@@ -987,7 +1422,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">CHTR</t>
+          <t xml:space="preserve">BMY</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000014272</t>
         </is>
       </c>
       <c r="E89">
@@ -997,7 +1437,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">TTWO</t>
+          <t xml:space="preserve">COF</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000927628</t>
         </is>
       </c>
       <c r="E90">
@@ -1007,7 +1452,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">WBD</t>
+          <t xml:space="preserve">PLD</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001045609</t>
         </is>
       </c>
       <c r="E91">
@@ -1017,37 +1467,57 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">LIN</t>
+          <t xml:space="preserve">PGR</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000080661</t>
         </is>
       </c>
       <c r="E92">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">APD</t>
+          <t xml:space="preserve">DHR</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000313616</t>
         </is>
       </c>
       <c r="E93">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHW</t>
+          <t xml:space="preserve">SPGI</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000064040</t>
         </is>
       </c>
       <c r="E94">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">FCX</t>
+          <t xml:space="preserve">CB</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000896159</t>
         </is>
       </c>
       <c r="E95">
@@ -1057,7 +1527,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">NEM</t>
+          <t xml:space="preserve">CVS</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000064803</t>
         </is>
       </c>
       <c r="E96">
@@ -1067,7 +1542,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">NUE</t>
+          <t xml:space="preserve">PH</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000076334</t>
         </is>
       </c>
       <c r="E97">
@@ -1077,27 +1557,42 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLD</t>
+          <t xml:space="preserve">MDT</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001613103</t>
         </is>
       </c>
       <c r="E98">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMT</t>
+          <t xml:space="preserve">VLO</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001035002</t>
         </is>
       </c>
       <c r="E99">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPG</t>
+          <t xml:space="preserve">MPC</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0001510295</t>
         </is>
       </c>
       <c r="E100">
@@ -1107,7 +1602,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">O</t>
+          <t xml:space="preserve">MO</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0000764180</t>
         </is>
       </c>
       <c r="E101">
@@ -1127,7 +1627,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Hypothetical weighted portfolio · 100-company demo</t>
+          <t xml:space="preserve">S&amp;P 500 coverage portfolio · top 100 companies</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1639,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Upload this workbook in Research Hub → Portfolio research. The Holdings sheet contains 100 company tickers and hypothetical weight_pct values totaling 100%. Select Weighted portfolio — supplied weight_pct in Allocation settings after import.</t>
+          <t xml:space="preserve">Upload this workbook in Research Hub → Portfolio research. The Holdings sheet contains 100 company tickers, their verified SEC CIKs and hypothetical weight_pct values totaling 100%. Select Weighted portfolio — supplied weight_pct in Allocation settings after import.</t>
         </is>
       </c>
     </row>
@@ -1163,65 +1663,101 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">This is a selected demonstration list, not an index, a representative market sample, actual holdings or an investment recommendation.</t>
+          <t xml:space="preserve">The 100 largest issuer holdings in the stored S&amp;P 500 coverage list, ranked by combined IVV holding weight as of 2026-09-11. Share classes are combined by SEC issuer. Portfolio allocations are fixed hypothetical examples, independent of IVV weights; this is a dated research demonstration, not an index portfolio or an investment recommendation.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hypothetical weights</t>
+          <t xml:space="preserve">Coverage membership</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed hypothetical weights: 5 companies at 5% each, 15 at 2%, 30 at 1%, and 50 at 0.3%, totaling 100%. These educational inputs are not derived from market prices, company fundamentals, an index, or actual holdings and are not investment recommendations.</t>
+          <t xml:space="preserve">sec-coverage-v1:ivv:2026-09-11:3e50096539317ce6</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Weight units</t>
+          <t xml:space="preserve">Membership source</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">weight_pct uses percentage points: 5 means 5%, and 0.3 means 0.3%. These are literal values. The remaining input fields are blank. Clear the weights to use your own company research list.</t>
+          <t xml:space="preserve">IVV holdings as of 2026-09-11; https://www.ishares.com/us/products/239726/ishares-core-s-p-500-etf/latest-holdings.csv</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dates</t>
+          <t xml:space="preserve">Company selection</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">The example analysis is a dated capture. Running research retrieves current available public evidence; results and coverage may differ.</t>
+          <t xml:space="preserve">The 100 largest issuer holdings in the active IVV S&amp;P 500 coverage source, ranked by combined published fund weight across share classes. Ties use combined holding market value, then ticker. Each SEC issuer appears once, represented by its largest share class. IVV holdings are a dated coverage proxy, not certified current index membership.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Limits</t>
+          <t xml:space="preserve">Hypothetical weights</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">The import supports at most 100 rows. Replace existing tickers before adding more. Cells contain literal values, with no formulas or macros.</t>
+          <t xml:space="preserve">Fixed hypothetical weights by demo order: the first 5 companies receive 5% each, the next 15 receive 2%, the next 30 receive 1%, and the remaining 50 receive 0.3%, totaling 100%. These educational amounts are fixed independently of source fund weights, prices and company fundamentals. They are not actual holdings, index weights or investment recommendations.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t xml:space="preserve">Weight units</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weight_pct uses percentage points: 5 means 5%, and 0.3 means 0.3%. These are literal hypothetical allocations, not the IVV weights used to select companies. Other than ticker, CIK and weight_pct, the input fields are blank. Clear the weights to use company counts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dates</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The example analysis is a dated capture. Running research retrieves current available public evidence; results and coverage may differ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limits</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The import supports at most 100 rows. Replace existing tickers before adding more. Cells contain literal values, with no formulas or macros.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Privacy</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t xml:space="preserve">Imported notes remain in your browser. Interactive research sends company identifiers, not private allocations or notes.</t>
         </is>

</xml_diff>